<commit_message>
Stage 8 review fixes: A-016
</commit_message>
<xml_diff>
--- a/output/archive/VellacombeData/Clients/DT18/VD-19-120/Delivery/Lot3/DT18_route-transfer_02Mar20.xlsx
+++ b/output/archive/VellacombeData/Clients/DT18/VD-19-120/Delivery/Lot3/DT18_route-transfer_02Mar20.xlsx
@@ -158,21 +158,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Clara Fenwick</author>
-  </authors>
-  <commentList>
-    <comment ref="A4" authorId="0" shapeId="0">
-      <text>
-        <t>Lot 3 release sign-off pending the Doventhar QC report.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -464,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -575,12 +560,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Caveat</t>
+          <t>Transfer scope</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Crystallisation needs the seed from the first lot. Doventhar's batch will need a fresh seed if the lot is run from a new supplier of the acid.</t>
+          <t>Confirm work-up conditions and intermediate release requirements against the original route-transfer record before follow-up preparation.</t>
         </is>
       </c>
     </row>
@@ -618,6 +603,18 @@
       <c r="D14" s="2" t="inlineStr">
         <is>
           <t>02/03/2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Firm</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Vellacombe Discovery Ltd, a Tarnovell company</t>
         </is>
       </c>
     </row>
@@ -636,7 +633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -654,24 +651,14 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Work-up</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>Procedure</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t>Scale (mmol)</t>
-        </is>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>Outcome</t>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Route-transfer note</t>
         </is>
       </c>
     </row>
@@ -683,17 +670,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Silica column, EtOAc/heptane gradient</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Recovery accepted for the first runs. Slow, and solvent-heavy on the larger scale.</t>
+          <t>Previous work-up for the shared intermediate. Consult the original route records for recovery details.</t>
         </is>
       </c>
     </row>
@@ -705,52 +682,19 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Ethanol/water, cool slowly from reflux, filter</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Replaces the column. Crystals filter cleanly. Purity gain is as good or better in the HPLC.</t>
+          <t>Replaced chromatography for the shared intermediate and supported the outsourced follow-up batch.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Crystallisation, scale-up</t>
+          <t>Comparison limits</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>As above, 3x volume</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Ran in Nottingham. Seeded, no oiling out.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7"/>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Route gate</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Passed. Shared intermediate goes through crystallisation for all the remaining members.</t>
+          <t>The delivery table reports final-compound isolated yields and purity; it does not quantify intermediate recovery or purity differences between work-ups.</t>
         </is>
       </c>
     </row>
@@ -1824,6 +1768,5 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>